<commit_message>
Add VJM Global competitor validation to USA-India opportunity workbook
Cross-checked the workbook against VJM Global's full sitemap (7,197 URLs).
4 existing P1/P2 CREATE recommendations (PE risk, DTAA/repatriation,
Virtual CFO, ECB/funding) have a live VJM equivalent — now marked in a
new Competitor Validation column. Added 3 new items surfaced by the
review: a SOC 1/SOC 2/SOX audit page (P2, CREATE), a supporting blog on
why US companies outsource accounting to India (P4, BLOG), and a
Delaware/California state-page test (P3, VALIDATE FIRST — VJM's own
state coverage skips the largest formation states, so flagged unproven
rather than recommended for a full rollout).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017QrsCL3x6BAaZApUGbbGXs
</commit_message>
<xml_diff>
--- a/content-ops/keyword-database/usa-research/AU_Corporate_USA_India_Page_Opportunities.xlsx
+++ b/content-ops/keyword-database/usa-research/AU_Corporate_USA_India_Page_Opportunities.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +53,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000B5394"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000B5394"/>
       <sz val="10"/>
     </font>
     <font>
@@ -62,7 +74,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +123,12 @@
         <bgColor rgb="00D0E0F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -138,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -173,7 +191,19 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -541,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
@@ -580,97 +610,121 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>IMPORTANT — what is and isn't verified:</t>
+          <t>UPDATE — VJM Global competitor sitemap review (added after initial delivery):</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>• Semrush returned a no_api_units error on every attempt across all 3 research batches (active subscription, insufficient API units) — no search volume, keyword difficulty, or ranking-position data could be pulled.</t>
+          <t>VJM Global is a direct India-entry competitor. Their full sitemap (7,197 URLs) was reviewed and cross-checked against this workbook. Result: 4 of our existing P1/P2 CREATE recommendations (PE Risk, DTAA/Repatriation, Virtual CFO, ECB/Funding) have a live VJM equivalent — marked in the new “Competitor Validation” column on the Master Classification sheet. 3 new items were added as a result (shown in blue text/fill throughout): a SOC 1/SOC 2/SOX audit page (P2, CREATE), a supporting blog on why US companies outsource accounting to India (P4, BLOG), and a narrow Delaware/California state-page test (P3, VALIDATE FIRST — VJM's own state coverage skips the biggest formation states, so this is flagged as unproven, not recommended for a full state-by-state rollout).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>• Every finding is WebSearch-observed: based on which competitor pages exist and rank for a query, not confirmed search volume. Confidence ratings (High/Moderate/Low, Observed/Inferred) reflect how much direct evidence backs each item — not a substitute for real volume data.</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>• No search volumes, keyword difficulty scores, or rankings have been invented anywhere in this workbook.</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT — what is and isn't verified:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Recommend re-running Semrush/Ahrefs organic_research and keyword_research on the P1 items once API access is restored, before committing production resources.</t>
+          <t>• Semrush returned a no_api_units error on every attempt across all 3 research batches (active subscription, insufficient API units) — no search volume, keyword difficulty, or ranking-position data could be pulled.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>• Ahrefs returned “Insufficient plan” on every endpoint tested, including zero-cost test calls — a separate, non-retryable blocker on the Ahrefs account itself.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Sheets in this workbook:</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>• Every finding is WebSearch-observed or, for the VJM addendum, sitemap-observed: based on which competitor pages exist and rank for a query, not confirmed search volume. Confidence ratings (High/Moderate/Low, Observed/Inferred) reflect how much direct evidence backs each item — not a substitute for real volume data.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>1. Master Classification — all 46 opportunities found, each classified CREATE / MERGE / BLOG / FAQ / DO NOT CREATE / VALIDATE FIRST, with overlap-risk notes against existing AU pages and the in-progress page.</t>
+          <t>• No search volumes, keyword difficulty scores, or rankings have been invented anywhere in this workbook.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2. Top Pages (Ranked) — the CREATE-classified standalone commercial/service pages, in priority order. Real evidence supports 18 opportunities, not padded to 30 — see the note on that sheet.</t>
+          <t>• Recommend re-running Semrush/Ahrefs organic_research and keyword_research on the P1 items once API access is restored, before committing production resources.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>3. Supporting Blog Topics — 30 blog/guide topics that support the commercial pages without cannibalizing them.</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>4. Comparison Pages — 10 decision-stage comparison pages, several flagged as sections rather than standalone until validated.</t>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Sheets in this workbook:</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>5. Industry Pages — evaluated 8 industry groupings (14 individual industries per the brief's list); only 2 have real supporting evidence. Not padded to 10 — see the note on that sheet.</t>
+          <t>1. Master Classification — all 49 opportunities found (46 original + 3 from the VJM addendum), each classified CREATE / MERGE / BLOG / FAQ / DO NOT CREATE / VALIDATE FIRST, with overlap-risk notes and a Competitor Validation column against AU's existing pages, the in-progress page, and VJM Global.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2. Top Pages (Ranked) — the CREATE-classified standalone commercial/service pages, in priority order. Real evidence supports 20 opportunities, not padded to 30 — see the note on that sheet. New items (16 and 20) are shown in blue.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Priority key: P1 = high commercial opportunity · P2 = strong supporting opportunity · P3 = informational opportunity · P4 = optional / lower priority / not recommended</t>
+          <t>3. Supporting Blog Topics — 31 blog/guide topics that support the commercial pages without cannibalizing them. Item 31 is new.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Color key: green = CREATE · yellow = BLOG · orange = FAQ · blue = MERGE · pink = VALIDATE FIRST · red = DO NOT CREATE</t>
+          <t>4. Comparison Pages — 10 decision-stage comparison pages, several flagged as sections rather than standalone until validated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>5. Industry Pages — evaluated 8 industry groupings (14 individual industries per the brief's list); only 2 have real supporting evidence. Not padded to 10 — see the note on that sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Priority key: P1 = high commercial opportunity · P2 = strong supporting opportunity · P3 = informational opportunity · P4 = optional / lower priority / not recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Color key: green = CREATE · yellow = BLOG · orange = FAQ · blue fill/text = MERGE or new item added from the VJM Global review · pink = VALIDATE FIRST · red = DO NOT CREATE</t>
         </is>
       </c>
     </row>
@@ -685,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -698,7 +752,8 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -754,6 +809,11 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
+          <t>Competitor Validation</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
           <t>Action</t>
         </is>
       </c>
@@ -809,7 +869,12 @@
           <t>Low — distinct from the existing FEMA filing page (post-incorporation compliance vs. this pre-incorporation/no-entity risk)</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>VJM Global runs a live page on this exact topic — validates real demand</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -866,7 +931,12 @@
           <t>Low — complements, doesn't duplicate, the existing transfer-pricing page</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -923,7 +993,12 @@
           <t>None — genuinely new territory</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -980,7 +1055,12 @@
           <t>Low — hub's DTAA mention is narrow; must cross-link not duplicate</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>VJM Global runs a live page on this exact topic — validates real demand</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1037,7 +1117,12 @@
           <t>Low — complements the existing generic regulatory-compliance page</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1094,7 +1179,12 @@
           <t>Low — sits before, and should link to, the in-progress entity-comparison page</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1151,7 +1241,12 @@
           <t>Low — /outsourcing mentions Virtual CFO generically; this is the US-specific commercial page for that service</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>VJM Global runs a live page on this exact topic — validates real demand</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1208,7 +1303,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1265,7 +1365,12 @@
           <t>Low — none of AU's pages address individual citizenship-status distinctions</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1322,7 +1427,12 @@
           <t>Moderate — must clearly differentiate from existing FEMA page; cross-link required</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1379,7 +1489,12 @@
           <t>Moderate — must explicitly distinguish from OIDAR page in the copy itself</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1436,7 +1551,12 @@
           <t>Low-moderate — differentiate audience clearly (accounting firms vs. the US company itself)</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1493,7 +1613,12 @@
           <t>Low-moderate — same FEMA/RBI family as existing page; must frame as funding-structure decision, not restate filings</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>VJM Global runs a live page on this exact topic — validates real demand</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1550,7 +1675,12 @@
           <t>Low-moderate — must link to and differentiate from generic /llp-in-india</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1607,7 +1737,12 @@
           <t>Low — complements /hr-services, doesn't duplicate it</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>CREATE</t>
         </is>
@@ -1664,7 +1799,12 @@
           <t>Low, but validate demand first — no observed competitor doing this exact combination</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>VALIDATE FIRST</t>
         </is>
@@ -1721,7 +1861,12 @@
           <t>Low, but validate demand first</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>VALIDATE FIRST</t>
         </is>
@@ -1778,7 +1923,12 @@
           <t>Moderate — add as FAQ on in-progress page or hub, not a new standalone page</t>
         </is>
       </c>
-      <c r="K19" s="8" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -1835,7 +1985,12 @@
           <t>Low — add a US-framed section/FAQ to the existing page rather than build new</t>
         </is>
       </c>
-      <c r="K20" s="8" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -1892,7 +2047,12 @@
           <t>Low-moderate — cross-link to OIDAR page</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -1949,7 +2109,12 @@
           <t>Moderate — mechanics already covered on existing how-to page; only build if framed as a discrete commercial service</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
         <is>
           <t>CREATE (see above)</t>
         </is>
@@ -2006,7 +2171,12 @@
           <t>Low — fold into compliance calendar page as a section/FAQ</t>
         </is>
       </c>
-      <c r="K23" s="8" t="inlineStr">
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -2063,7 +2233,12 @@
           <t>Low — fold into compliance calendar page</t>
         </is>
       </c>
-      <c r="K24" s="8" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -2120,7 +2295,12 @@
           <t>Low — add as a section to the existing FEMA page</t>
         </is>
       </c>
-      <c r="K25" s="8" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -2177,7 +2357,12 @@
           <t>Low, but time-sensitive — publish promptly or skip</t>
         </is>
       </c>
-      <c r="K26" s="9" t="inlineStr">
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -2234,7 +2419,12 @@
           <t>Low — niche, lower priority unless AU wants a BFSI focus</t>
         </is>
       </c>
-      <c r="K27" s="9" t="inlineStr">
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -2291,7 +2481,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="K28" s="9" t="inlineStr">
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L28" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -2348,7 +2543,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="K29" s="9" t="inlineStr">
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -2405,7 +2605,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="K30" s="9" t="inlineStr">
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L30" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -2462,7 +2667,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="K31" s="9" t="inlineStr">
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -2519,7 +2729,12 @@
           <t>Low — cross-link to PE-risk page</t>
         </is>
       </c>
-      <c r="K32" s="9" t="inlineStr">
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L32" s="9" t="inlineStr">
         <is>
           <t>BLOG</t>
         </is>
@@ -2576,7 +2791,12 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="K33" s="8" t="inlineStr">
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L33" s="8" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -2633,7 +2853,12 @@
           <t>Low — fold into WOS vs JV page as FAQ</t>
         </is>
       </c>
-      <c r="K34" s="8" t="inlineStr">
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L34" s="8" t="inlineStr">
         <is>
           <t>FAQ</t>
         </is>
@@ -2690,7 +2915,12 @@
           <t>High — would duplicate /india-entry-for-saas-companies and /oidar-gst-registration-india</t>
         </is>
       </c>
-      <c r="K35" s="10" t="inlineStr">
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L35" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -2747,7 +2977,12 @@
           <t>High — direct duplicate</t>
         </is>
       </c>
-      <c r="K36" s="10" t="inlineStr">
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L36" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -2804,7 +3039,12 @@
           <t>Moderate — low strategic fit for an advisory firm</t>
         </is>
       </c>
-      <c r="K37" s="10" t="inlineStr">
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L37" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -2861,7 +3101,12 @@
           <t>Low overlap, but requires an explicit scope decision from AU on whether to offer immigration-adjacent content</t>
         </is>
       </c>
-      <c r="K38" s="7" t="inlineStr">
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
         <is>
           <t>VALIDATE FIRST</t>
         </is>
@@ -2918,7 +3163,12 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="K39" s="10" t="inlineStr">
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L39" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -2975,7 +3225,12 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="K40" s="10" t="inlineStr">
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L40" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -3032,7 +3287,12 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="K41" s="10" t="inlineStr">
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L41" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -3089,7 +3349,12 @@
           <t>High — direct duplicate</t>
         </is>
       </c>
-      <c r="K42" s="10" t="inlineStr">
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L42" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -3146,7 +3411,12 @@
           <t>High — direct duplicate of in-progress work</t>
         </is>
       </c>
-      <c r="K43" s="11" t="inlineStr">
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L43" s="11" t="inlineStr">
         <is>
           <t>MERGE</t>
         </is>
@@ -3203,7 +3473,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="K44" s="10" t="inlineStr">
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L44" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE</t>
         </is>
@@ -3260,7 +3535,12 @@
           <t>High — exists already</t>
         </is>
       </c>
-      <c r="K45" s="10" t="inlineStr">
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L45" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE (consider refreshing given SERP crowding)</t>
         </is>
@@ -3317,7 +3597,12 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="K46" s="11" t="inlineStr">
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L46" s="11" t="inlineStr">
         <is>
           <t>MERGE</t>
         </is>
@@ -3374,9 +3659,200 @@
           <t>High — direct duplicate</t>
         </is>
       </c>
-      <c r="K47" s="10" t="inlineStr">
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>Not directly checked against VJM Global's sitemap</t>
+        </is>
+      </c>
+      <c r="L47" s="10" t="inlineStr">
         <is>
           <t>DO NOT CREATE (already exists)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>SOC 1 / SOC 2 / SOX Audit &amp; Controls Assurance for US Companies' Indian Operations</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>/india-entry-for-us-companies/soc-sox-audit-controls-india</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>SOC 2 audit India for US company</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>SOC 1 audit India; SOX controls assurance Indian subsidiary; SOC 2 compliance India outsourcing; financial controls audit Indian subsidiary</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Commercial, service page</t>
+        </is>
+      </c>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>US parent-company finance/compliance teams needing controls assurance over Indian operations or an India-based outsourced team</t>
+        </is>
+      </c>
+      <c r="H48" s="12" t="inlineStr">
+        <is>
+          <t>Service landing page</t>
+        </is>
+      </c>
+      <c r="I48" s="12" t="inlineStr">
+        <is>
+          <t>VJM Global runs 3 dedicated pages on this exact topic; AU currently only lists 'SOX &amp; Controls Assurance' as a bullet on the generic /services/accounting-assurance page — no dedicated US-facing page</t>
+        </is>
+      </c>
+      <c r="J48" s="12" t="inlineStr">
+        <is>
+          <t>Low-moderate — differentiate from the generic assurance page by framing as US-parent oversight of Indian subsidiary/outsourced-operations controls</t>
+        </is>
+      </c>
+      <c r="K48" s="12" t="inlineStr">
+        <is>
+          <t>New finding — VJM Global runs 3 dedicated pages (SOC 1, SOC 2, SOX) on this exact topic</t>
+        </is>
+      </c>
+      <c r="L48" s="13" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>Why US Companies/Startups Outsource Accounting to India</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>/blog/why-us-companies-outsource-accounting-to-india</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>why US companies outsource accounting to India</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>benefits of outsourcing accounting to India; US CPA firms outsourcing India; cost savings accounting outsourcing India</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Informational, top-of-funnel</t>
+        </is>
+      </c>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>US companies/CPA firms evaluating whether to outsource at all</t>
+        </is>
+      </c>
+      <c r="H49" s="12" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="I49" s="12" t="inlineStr">
+        <is>
+          <t>VJM Global runs this exact framing (2 posts: companies + startups variants) feeding their commercial accounting-outsourcing page; AU has the commercial page (/accounting-outsourcing-firm-for-united-states-cpas-firm) but no supporting top-of-funnel content driving into it</t>
+        </is>
+      </c>
+      <c r="J49" s="12" t="inlineStr">
+        <is>
+          <t>Low — supports, doesn't duplicate, the existing commercial page</t>
+        </is>
+      </c>
+      <c r="K49" s="12" t="inlineStr">
+        <is>
+          <t>New finding — VJM Global's content-funnel pattern (2 posts feeding their outsourcing page); AU has the commercial page but no equivalent top-of-funnel content</t>
+        </is>
+      </c>
+      <c r="L49" s="14" t="inlineStr">
+        <is>
+          <t>BLOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>Register a Company in India from Delaware / California (state-specific test pages)</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>/india-entry-for-us-companies/register-company-india-from-delaware  (+ ...-from-california)</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>register company in India from Delaware</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>start business in India from California; India company registration for Delaware companies</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Commercial, narrow geographic</t>
+        </is>
+      </c>
+      <c r="G50" s="12" t="inlineStr">
+        <is>
+          <t>US companies incorporated specifically in Delaware or California researching India entry</t>
+        </is>
+      </c>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>Landing page (programmatic test)</t>
+        </is>
+      </c>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>VJM Global runs a state-level template, but skips the states that actually matter most for company formation — treat as unproven, test narrowly rather than replicate their list</t>
+        </is>
+      </c>
+      <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>Low — genuinely new page type for AU; no existing state-level content to conflict with</t>
+        </is>
+      </c>
+      <c r="K50" s="12" t="inlineStr">
+        <is>
+          <t>New finding — VJM runs a start-business-[state]-india template for 6 states (California, Arizona, Colorado, Illinois, Wisconsin, Alabama), but conspicuously NOT Texas, Florida, New York, or Delaware — the states with the largest company-formation volume. Reads as a thin programmatic sweep, not a proven-demand bet.</t>
+        </is>
+      </c>
+      <c r="L50" s="15" t="inlineStr">
+        <is>
+          <t>VALIDATE FIRST</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3407,10 +3883,10 @@
     <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>You asked for a Top 30. Real, evidence-backed standalone-page opportunities support 18, not 30 — padding to 30 would mean including thin, duplicate, or unvalidated items, which fails your own Section 28 Final Filter ("would a US company genuinely search this separately, and can AU genuinely help"). Items 17-18 are flagged VALIDATE FIRST rather than CREATE: real regulatory hooks exist, but no competitor evidence confirms a US-company-specific search cluster for these two verticals — recommend a quick Semrush/Ahrefs check once API access is restored before committing to them. 12 further blog/FAQ-tier opportunities exist beyond these 18 — see the Supporting Blog Topics sheet.</t>
+    <row r="1" ht="75" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>You asked for a Top 30. Real, evidence-backed standalone-page opportunities support 20 (18 from the original research + 2 added after reviewing VJM Global's competitor sitemap) — not 30. Padding to 30 would mean including thin, duplicate, or unvalidated items, which fails your own Section 28 Final Filter ("would a US company genuinely search this separately, and can AU genuinely help"). Item 16 (SOC/SOX) and item 20 (Delaware/California state test) are new additions from the VJM Global sitemap review. Items 18-19 (Manufacturing, Fintech) remain flagged VALIDATE FIRST as before: real regulatory hooks, but no confirmed US-company-specific search cluster. Item 20 is also VALIDATE FIRST — VJM's own state-page coverage is inconsistent (misses the largest formation states), so treat it as an unproven pattern to test narrowly, not a validated opportunity. 12 further blog/FAQ-tier opportunities exist beyond these 20 — see the Supporting Blog Topics sheet.</t>
         </is>
       </c>
     </row>
@@ -4297,57 +4773,57 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>India's New Labour Codes: What US Companies with Indian Employees Need to Know</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>/blog/india-labour-codes-2026-us-companies</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>India Labour Codes 2026 US companies</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>new labour codes India impact foreign employers · India labour law changes 2026 · four labour codes India explained</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Informational, timely</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>US companies with Indian employees (subsidiary or EOR)</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Blog / regulatory explainer</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>Timely, real regulatory change (effective Nov 2025) with dedicated competitor coverage; freshness advantage available now</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>/hr-services</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>EOR vs subsidiary page</t>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>SOC 1 / SOC 2 / SOX Audit &amp; Controls Assurance for US Companies' Indian Operations</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>/india-entry-for-us-companies/soc-sox-audit-controls-india</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>SOC 2 audit India for US company</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>SOC 1 audit India · SOX controls assurance Indian subsidiary · SOC 2 compliance India outsourcing · financial controls audit Indian subsidiary</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Commercial, service page</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>US parent-company finance/compliance teams needing controls assurance over Indian operations or an India-based outsourced team</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>Service landing page</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>VJM Global runs 3 dedicated pages (SOC 1, SOC 2, SOX) on this exact topic — new finding from the competitor sitemap review; AU only has a passing bullet mention today</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>/services/accounting-assurance, Virtual CFO page</t>
+        </is>
+      </c>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>Virtual CFO page, Ind AS vs US GAAP page, hub page</t>
         </is>
       </c>
     </row>
@@ -4357,52 +4833,52 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>India Market Entry for US Manufacturers: PLI Scheme &amp; China+1 Opportunity</t>
+          <t>India's New Labour Codes: What US Companies with Indian Employees Need to Know</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>/india-entry-for-us-companies/manufacturing-india-entry-pli-scheme</t>
+          <t>/blog/india-labour-codes-2026-us-companies</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>US manufacturing company India expansion</t>
+          <t>India Labour Codes 2026 US companies</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>PLI scheme eligibility foreign company · China plus one India manufacturing · US manufacturer India subsidiary · India manufacturing FDI</t>
+          <t>new labour codes India impact foreign employers · India labour law changes 2026 · four labour codes India explained</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Strategic/commercial</t>
+          <t>Informational, timely</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>US manufacturing/industrial companies evaluating India as a production base</t>
+          <t>US companies with Indian employees (subsidiary or EOR)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Guide page</t>
+          <t>Blog / regulatory explainer</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>VALIDATE FIRST — real regulatory hook (PLI) but no observed competitor doing this exact combination; inferred, not confirmed, opportunity</t>
+          <t>Timely, real regulatory change (effective Nov 2025) with dedicated competitor coverage; freshness advantage available now</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Hub page</t>
+          <t>/hr-services</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Hub page</t>
+          <t>EOR vs subsidiary page</t>
         </is>
       </c>
     </row>
@@ -4412,50 +4888,160 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
+          <t>India Market Entry for US Manufacturers: PLI Scheme &amp; China+1 Opportunity</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>/india-entry-for-us-companies/manufacturing-india-entry-pli-scheme</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>US manufacturing company India expansion</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>PLI scheme eligibility foreign company · China plus one India manufacturing · US manufacturer India subsidiary · India manufacturing FDI</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Strategic/commercial</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>US manufacturing/industrial companies evaluating India as a production base</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Guide page</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>VALIDATE FIRST — real regulatory hook (PLI) but no observed competitor doing this exact combination; inferred, not confirmed, opportunity</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Hub page</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Hub page</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
           <t>India Market Entry for US Fintech Companies: RBI Licensing &amp; NBFC Setup</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>/india-entry-for-us-companies/fintech-india-entry-rbi-licensing</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>US fintech company India expansion</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>RBI payment aggregator license foreign company · NBFC setup foreign company India · fintech regulatory sandbox India · digital lending guidelines India</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Strategic/commercial</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>US fintech/payments companies evaluating India entry</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>Guide page</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>VALIDATE FIRST — real regulatory stack but no observed competitor framing it for US companies specifically; inferred opportunity</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>Hub page</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Hub page</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Register a Company in India from Delaware / California (state-specific test)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>/india-entry-for-us-companies/register-company-india-from-delaware</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>register company in India from Delaware</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>start business in India from California · India company registration for Delaware companies</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Commercial, narrow geographic</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>US companies incorporated specifically in Delaware or California researching India entry</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Landing page (programmatic test — 2 pages only)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>VALIDATE FIRST — VJM runs this template for 6 states but skips Texas/Florida/New York/Delaware, the states with the most company formations, suggesting unproven demand; test Delaware + California only, don't replicate their full list</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Hub page</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>Hub page</t>
         </is>
@@ -4475,7 +5061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5727,6 +6313,46 @@
       <c r="H31" s="5" t="inlineStr">
         <is>
           <t>Recurring named constraint across NRI/OCI/foreign-national comparison content — natural 'if not OPC, then what' follow-on</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Why US Companies and US Startups Outsource Accounting to India</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>/blog/why-us-companies-outsource-accounting-to-india</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>why US companies outsource accounting to India</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Informational, top-of-funnel</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>US companies/CPA firms evaluating whether to outsource at all</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>/accounting-outsourcing-firm-for-united-states-cpas-firm</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>New finding from VJM Global's sitemap — they run this exact framing as 2 posts feeding their commercial outsourcing page; AU has the commercial page but no supporting top-of-funnel content</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6731,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="75" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>You asked for a Top 10. Of 14 industries evaluated (SaaS/AI/software/IT/technology counted together, per the brief's own category 18 list), only 2 (Manufacturing, Fintech) have a real, distinct regulatory hook that isn't yet captured by any observed competitor as a US-company-specific page — and even those are flagged VALIDATE FIRST, not a confirmed CREATE. The other 6 evaluated verticals show no evidence of genuine US-company-specific search demand beyond AU's existing generic pages. Recommending 10 would mean inventing demand for 4+ industries with no supporting evidence, which fails your own Section 28 filter and Section 18 instruction ("do not create industry pages merely because an industry exists"). Full reasoning per industry below.</t>
         </is>

</xml_diff>